<commit_message>
BasicsdOfANN and MolecularRepresentations can now be run in Google Colab
</commit_message>
<xml_diff>
--- a/Molecules-data/smiles_prop_3xtr_WithTokenMol.xlsx
+++ b/Molecules-data/smiles_prop_3xtr_WithTokenMol.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Smiles</t>
   </si>
@@ -40,10 +40,7 @@
     <t>ROMol</t>
   </si>
   <si>
-    <t>O=Cc1cc2cccc3c2n(c1=O)CCC3</t>
-  </si>
-  <si>
-    <t>['O', '=', 'C', 'c', '1', 'c', 'c', '2', 'c', 'c', 'c', 'c', '3', 'c', '2', 'n', '(', 'c', '1', '=', 'O', ')', 'C', 'C', 'C', '3']</t>
+    <t>['O', '=', 'C', '(', 'N', '[C@@H]', '1', 'C', 'C', 'S', 'C', '1', '=', 'O', ')', 'c', '1', 'c', 'c', 'c', 'c', '(', 'Br', ')', 'c', '1']</t>
   </si>
   <si>
     <t>[[1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
@@ -51,34 +48,27 @@
  [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
  [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
@@ -100,113 +90,93 @@
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]]</t>
   </si>
   <si>
-    <t>CC(C)(C)[C@H]1CCc2c(sc(NC(=O)c3ccc4c(c3)OCO4)c2C(N)=O)C1</t>
-  </si>
-  <si>
-    <t>['C', 'C', '(', 'C', ')', '(', 'C', ')', '[C@H]', '1', 'C', 'C', 'c', '2', 'c', '(', 's', 'c', '(', 'N', 'C', '(', '=', 'O', ')', 'c', '3', 'c', 'c', 'c', '4', 'c', '(', 'c', '3', ')', 'O', 'C', 'O', '4', ')', 'c', '2', 'C', '(', 'N', ')', '=', 'O', ')', 'C', '1']</t>
+    <t>['C', '[C@@H]', '1', 'C', 'C', 'C', 'C', '[C@H]', '1', 'N', 'S', '(', '=', 'O', ')', '(', '=', 'O', ')', 'c', '1', 'c', 'c', 'c', '(', 'S', '(', '=', 'O', ')', '(', '=', 'O', ')', 'N', '2', 'C', 'C', 'C', 'C', '2', ')', 'c', 'c', '1']</t>
   </si>
   <si>
     <t>[[0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0]
+ [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]]</t>
-  </si>
-  <si>
-    <t>Cc1ccc(S[C@@H](C)C(=O)Nc2cccc(C(F)(F)F)c2)cc1</t>
-  </si>
-  <si>
-    <t>['C', 'c', '1', 'c', 'c', 'c', '(', 'S', '[C@@H]', '(', 'C', ')', 'C', '(', '=', 'O', ')', 'N', 'c', '2', 'c', 'c', 'c', 'c', '(', 'C', '(', 'F', ')', '(', 'F', ')', 'F', ')', 'c', '2', ')', 'c', 'c', '1']</t>
-  </si>
-  <si>
-    <t>[[0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
- [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]]</t>
+  </si>
+  <si>
+    <t>['O', '=', '[N+]', '(', '[O-]', ')', 'c', '1', 'c', 'c', 'c', '2', 'n', 'n', 'n', '(', 'O', 'C', 'c', '3', 'c', 'c', 'c', '(', 'Br', ')', 'c', 'c', '3', ')', 'c', '2', 'c', '1']</t>
+  </si>
+  <si>
+    <t>[[1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [1 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1]
  [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 1]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 1 0 0 0 0 0 0 0 0 0 0 0 0]
- [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 0 0 0 1 0 0 0 0]
+ [0 0 0 0 0 0 0 0 0 1 0 0 0 0 0 0 0]
+ [0 0 0 0 0 0 1 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
  [0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0]
@@ -275,9 +245,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2857500</xdr:colOff>
+      <xdr:colOff>2857143</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>2857500</xdr:rowOff>
+      <xdr:rowOff>2857143</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -295,7 +265,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4267200" y="190500"/>
-          <a:ext cx="2857500" cy="2857500"/>
+          <a:ext cx="2857143" cy="2857143"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -313,9 +283,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2857500</xdr:colOff>
+      <xdr:colOff>2857143</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>2857500</xdr:rowOff>
+      <xdr:rowOff>2857143</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -332,8 +302,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4267200" y="4000500"/>
-          <a:ext cx="2857500" cy="2857500"/>
+          <a:off x="4267200" y="3048000"/>
+          <a:ext cx="2857143" cy="2857143"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -351,9 +321,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2857500</xdr:colOff>
+      <xdr:colOff>2857143</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>2857500</xdr:rowOff>
+      <xdr:rowOff>2857143</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -370,8 +340,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4267200" y="7810500"/>
-          <a:ext cx="2857500" cy="2857500"/>
+          <a:off x="4267200" y="5905500"/>
+          <a:ext cx="2857143" cy="2857143"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -671,7 +641,7 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="50.7109375" customWidth="1"/>
+    <col min="8" max="8" width="42.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -700,73 +670,55 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="300" customHeight="1">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" ht="225" customHeight="1">
+      <c r="B2">
+        <v>298.96156166</v>
+      </c>
+      <c r="C2">
+        <v>2.211</v>
+      </c>
+      <c r="D2">
+        <v>46.17</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
-        <v>213.078978592</v>
-      </c>
-      <c r="C2">
-        <v>1.7602</v>
-      </c>
-      <c r="D2">
-        <v>39.07</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="225" customHeight="1">
+      <c r="B3">
+        <v>386.133399312</v>
+      </c>
+      <c r="C3">
+        <v>2.3281</v>
+      </c>
+      <c r="D3">
+        <v>83.55</v>
+      </c>
+      <c r="F3" t="s">
         <v>10</v>
       </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="300" customHeight="1">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
-        <v>400.145678248</v>
-      </c>
-      <c r="C3">
-        <v>3.979</v>
-      </c>
-      <c r="D3">
-        <v>90.65000000000001</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+    <row r="4" spans="1:8" ht="225" customHeight="1">
+      <c r="B4">
+        <v>347.985802248</v>
+      </c>
+      <c r="C4">
+        <v>2.7308</v>
+      </c>
+      <c r="D4">
+        <v>83.08</v>
+      </c>
+      <c r="F4" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="300" customHeight="1">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4">
-        <v>339.090469792</v>
-      </c>
-      <c r="C4">
-        <v>5.13312</v>
-      </c>
-      <c r="D4">
-        <v>29.1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>